<commit_message>
Day 1 Wch first session
</commit_message>
<xml_diff>
--- a/pages/Worlds_2023/Master.xlsx
+++ b/pages/Worlds_2023/Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\Worlds_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C0969FD-D9CC-40BE-A514-FE2FA115F2E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B76B51-B495-4FCB-8E71-CA13A399AA34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="252" yWindow="0" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="50">
   <si>
     <t>FileName</t>
   </si>
@@ -142,6 +142,39 @@
   </si>
   <si>
     <t>https://youtu.be/EMGzc8kcDwo</t>
+  </si>
+  <si>
+    <t>3_8_AG_TP_Q</t>
+  </si>
+  <si>
+    <t>3_8_BB_IP_Q</t>
+  </si>
+  <si>
+    <t>3_8_CS_TP_Q</t>
+  </si>
+  <si>
+    <t>3_8_EA_TS_Q</t>
+  </si>
+  <si>
+    <t>3_8_NK_TP_Q</t>
+  </si>
+  <si>
+    <t>3_8_RP_TS_Q</t>
+  </si>
+  <si>
+    <t>3_8_SF_TS_Q</t>
+  </si>
+  <si>
+    <t>3_8_TS_TP_Q</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xdnrdvLVwME</t>
+  </si>
+  <si>
+    <t>https://youtu.be/63pks-zGKqc</t>
+  </si>
+  <si>
+    <t>https://youtu.be/cEuhXhaq-rM</t>
   </si>
 </sst>
 </file>
@@ -459,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B27"/>
+  <dimension ref="A1:B35"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
@@ -676,6 +709,70 @@
         <v>33</v>
       </c>
     </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>39</v>
+      </c>
+      <c r="B28" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>40</v>
+      </c>
+      <c r="B29" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>41</v>
+      </c>
+      <c r="B30" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>42</v>
+      </c>
+      <c r="B31" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>43</v>
+      </c>
+      <c r="B32" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>44</v>
+      </c>
+      <c r="B33" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>45</v>
+      </c>
+      <c r="B34" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>46</v>
+      </c>
+      <c r="B35" t="s">
+        <v>49</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
day 1 second session
</commit_message>
<xml_diff>
--- a/pages/Worlds_2023/Master.xlsx
+++ b/pages/Worlds_2023/Master.xlsx
@@ -8,24 +8,35 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\Worlds_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10B76B51-B495-4FCB-8E71-CA13A399AA34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC62461-5B50-43C3-8EA7-59F05097D7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="252" yWindow="0" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9504" yWindow="0" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
   <si>
     <t>FileName</t>
   </si>
@@ -175,6 +186,24 @@
   </si>
   <si>
     <t>https://youtu.be/cEuhXhaq-rM</t>
+  </si>
+  <si>
+    <t>3_8_EA_TS_R1</t>
+  </si>
+  <si>
+    <t>3_8_SF_TS_R1</t>
+  </si>
+  <si>
+    <t>3_8_RP_TS_R1</t>
+  </si>
+  <si>
+    <t>3_8_BB_IP_F</t>
+  </si>
+  <si>
+    <t>https://youtu.be/jN5BZ0WpgDc</t>
+  </si>
+  <si>
+    <t>https://youtu.be/Xj1osb8m4ik</t>
   </si>
 </sst>
 </file>
@@ -492,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
@@ -773,6 +802,38 @@
         <v>49</v>
       </c>
     </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>51</v>
+      </c>
+      <c r="B37" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>52</v>
+      </c>
+      <c r="B38" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>53</v>
+      </c>
+      <c r="B39" t="s">
+        <v>54</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
day 2 morning session
</commit_message>
<xml_diff>
--- a/pages/Worlds_2023/Master.xlsx
+++ b/pages/Worlds_2023/Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\Worlds_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFC62461-5B50-43C3-8EA7-59F05097D7D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3925F22-DAD4-4EA5-9D2F-CD276C645ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9504" yWindow="0" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="10920" yWindow="0" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
   <si>
     <t>FileName</t>
   </si>
@@ -204,6 +204,18 @@
   </si>
   <si>
     <t>https://youtu.be/Xj1osb8m4ik</t>
+  </si>
+  <si>
+    <t>4_8_BB_TP_Q</t>
+  </si>
+  <si>
+    <t>4_8_ES_TP_Q</t>
+  </si>
+  <si>
+    <t>4_8_MD_TP_Q</t>
+  </si>
+  <si>
+    <t>https://youtu.be/TWHI0YDcNzk</t>
   </si>
 </sst>
 </file>
@@ -521,7 +533,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B39"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
@@ -834,6 +846,30 @@
         <v>54</v>
       </c>
     </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>56</v>
+      </c>
+      <c r="B40" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>57</v>
+      </c>
+      <c r="B41" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>58</v>
+      </c>
+      <c r="B42" t="s">
+        <v>59</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
day 2 evening sessions
</commit_message>
<xml_diff>
--- a/pages/Worlds_2023/Master.xlsx
+++ b/pages/Worlds_2023/Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\Worlds_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3925F22-DAD4-4EA5-9D2F-CD276C645ED9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7048F9F-FEF7-4ABE-93C9-58E4F3C5D537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10920" yWindow="0" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12504" yWindow="0" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="65">
   <si>
     <t>FileName</t>
   </si>
@@ -216,6 +216,21 @@
   </si>
   <si>
     <t>https://youtu.be/TWHI0YDcNzk</t>
+  </si>
+  <si>
+    <t>4_8_AG_TP_R1</t>
+  </si>
+  <si>
+    <t>4_8_NK_TP_R1</t>
+  </si>
+  <si>
+    <t>4_8_TS_TP_R1</t>
+  </si>
+  <si>
+    <t>4_8_CS_TP_R1</t>
+  </si>
+  <si>
+    <t>https://youtu.be/_Jbk5M_6jbU</t>
   </si>
 </sst>
 </file>
@@ -533,7 +548,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B42"/>
+  <dimension ref="A1:B46"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
@@ -870,6 +885,38 @@
         <v>59</v>
       </c>
     </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>60</v>
+      </c>
+      <c r="B43" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>62</v>
+      </c>
+      <c r="B45" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>63</v>
+      </c>
+      <c r="B46" t="s">
+        <v>64</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
morning session day 3
</commit_message>
<xml_diff>
--- a/pages/Worlds_2023/Master.xlsx
+++ b/pages/Worlds_2023/Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\Worlds_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7048F9F-FEF7-4ABE-93C9-58E4F3C5D537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{739B8F28-9C6D-47E2-A2ED-C932223EFA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12504" yWindow="0" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6972" yWindow="4692" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="74">
   <si>
     <t>FileName</t>
   </si>
@@ -231,6 +231,33 @@
   </si>
   <si>
     <t>https://youtu.be/_Jbk5M_6jbU</t>
+  </si>
+  <si>
+    <t>5_8_SD_SP_Q</t>
+  </si>
+  <si>
+    <t>5_8_SD_SP_R16</t>
+  </si>
+  <si>
+    <t>5_8_ES_TP_R1</t>
+  </si>
+  <si>
+    <t>5_8_MD_TP_R1</t>
+  </si>
+  <si>
+    <t>5_8_AW_TP_R1</t>
+  </si>
+  <si>
+    <t>5_8_BB_TP_R1</t>
+  </si>
+  <si>
+    <t>https://youtu.be/SPSduTrQse8</t>
+  </si>
+  <si>
+    <t>https://youtu.be/6OcTAWUlbR0</t>
+  </si>
+  <si>
+    <t>https://youtu.be/H-KDj5p95sM</t>
   </si>
 </sst>
 </file>
@@ -548,7 +575,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B46"/>
+  <dimension ref="A1:B52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
@@ -917,6 +944,54 @@
         <v>64</v>
       </c>
     </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>65</v>
+      </c>
+      <c r="B47" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>66</v>
+      </c>
+      <c r="B48" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>67</v>
+      </c>
+      <c r="B49" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>68</v>
+      </c>
+      <c r="B50" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>69</v>
+      </c>
+      <c r="B51" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>70</v>
+      </c>
+      <c r="B52" t="s">
+        <v>73</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
day 4 morning session
</commit_message>
<xml_diff>
--- a/pages/Worlds_2023/Master.xlsx
+++ b/pages/Worlds_2023/Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\Worlds_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{739B8F28-9C6D-47E2-A2ED-C932223EFA4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E40E2B-4046-4710-8021-EE1B4832F2AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6972" yWindow="4692" windowWidth="9612" windowHeight="12504" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1536" yWindow="1008" windowWidth="11256" windowHeight="11952" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="92">
   <si>
     <t>FileName</t>
   </si>
@@ -258,6 +258,60 @@
   </si>
   <si>
     <t>https://youtu.be/H-KDj5p95sM</t>
+  </si>
+  <si>
+    <t>5_8_ES_TP_F</t>
+  </si>
+  <si>
+    <t>5_8_MD_TP_F</t>
+  </si>
+  <si>
+    <t>5_8_AW_TP_F</t>
+  </si>
+  <si>
+    <t>5_8_BB_TP_F</t>
+  </si>
+  <si>
+    <t>https://youtu.be/DmxsxS_-gJw</t>
+  </si>
+  <si>
+    <t>5_8_AG_TP_F</t>
+  </si>
+  <si>
+    <t>5_8_CS_TP_F</t>
+  </si>
+  <si>
+    <t>5_8_NK_TP_F</t>
+  </si>
+  <si>
+    <t>5_8_TS_TP_F</t>
+  </si>
+  <si>
+    <t>https://youtu.be/xiW4Wx0YtRM</t>
+  </si>
+  <si>
+    <t>5_8_EA_KE_R16</t>
+  </si>
+  <si>
+    <t>https://youtu.be/79I-5x67Fo8</t>
+  </si>
+  <si>
+    <t>6_8_EA_KE_QF</t>
+  </si>
+  <si>
+    <t>https://youtu.be/seNzi2AlEDg</t>
+  </si>
+  <si>
+    <t>6_8_TS_IP_Q</t>
+  </si>
+  <si>
+    <t>https://youtu.be/kMm4Y9rzpyc</t>
+  </si>
+  <si>
+    <t>https://youtu.be/k380NhorOQg</t>
+  </si>
+  <si>
+    <t>6_8_CS_OM_SC</t>
   </si>
 </sst>
 </file>
@@ -575,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B52"/>
+  <dimension ref="A1:B64"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
@@ -992,6 +1046,102 @@
         <v>73</v>
       </c>
     </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>74</v>
+      </c>
+      <c r="B53" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>75</v>
+      </c>
+      <c r="B54" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>76</v>
+      </c>
+      <c r="B55" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>77</v>
+      </c>
+      <c r="B56" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>81</v>
+      </c>
+      <c r="B57" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>80</v>
+      </c>
+      <c r="B58" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>82</v>
+      </c>
+      <c r="B59" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>79</v>
+      </c>
+      <c r="B60" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>84</v>
+      </c>
+      <c r="B61" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>86</v>
+      </c>
+      <c r="B62" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>88</v>
+      </c>
+      <c r="B63" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>91</v>
+      </c>
+      <c r="B64" t="s">
+        <v>90</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
day 4 evening session
</commit_message>
<xml_diff>
--- a/pages/Worlds_2023/Master.xlsx
+++ b/pages/Worlds_2023/Master.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SamB\CNZPD\pages\Worlds_2023\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E40E2B-4046-4710-8021-EE1B4832F2AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA95B36-3733-4002-8286-D740A43A0461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1536" yWindow="1008" windowWidth="11256" windowHeight="11952" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="768" yWindow="636" windowWidth="11472" windowHeight="11868" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="102">
   <si>
     <t>FileName</t>
   </si>
@@ -308,10 +308,40 @@
     <t>https://youtu.be/kMm4Y9rzpyc</t>
   </si>
   <si>
-    <t>https://youtu.be/k380NhorOQg</t>
-  </si>
-  <si>
-    <t>6_8_CS_OM_SC</t>
+    <t>https://youtu.be/L9T4gRnuJOk</t>
+  </si>
+  <si>
+    <t>6_8_CS_OM_Tempo</t>
+  </si>
+  <si>
+    <t>6_8_CS_OM_Scratch</t>
+  </si>
+  <si>
+    <t>6_8_CS_OM_Elim</t>
+  </si>
+  <si>
+    <t>6_8_CS_OM_Points</t>
+  </si>
+  <si>
+    <t>https://youtu.be/X4RrOi6bw9o</t>
+  </si>
+  <si>
+    <t>https://youtu.be/bIvxXxZ2HzU</t>
+  </si>
+  <si>
+    <t>https://youtu.be/UQDv36972yw</t>
+  </si>
+  <si>
+    <t>6_8_EA_KE_SF</t>
+  </si>
+  <si>
+    <t>6_8_EA_KE_F</t>
+  </si>
+  <si>
+    <t>https://youtu.be/wZ-3ZGLHlJQ</t>
+  </si>
+  <si>
+    <t>https://youtu.be/ENVeTeTwSj0</t>
   </si>
 </sst>
 </file>
@@ -629,7 +659,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B64"/>
+  <dimension ref="A1:B69"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="26.109375" bestFit="1" customWidth="1"/>
@@ -1136,10 +1166,50 @@
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B64" t="s">
         <v>90</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>91</v>
+      </c>
+      <c r="B65" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>93</v>
+      </c>
+      <c r="B66" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>94</v>
+      </c>
+      <c r="B67" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>98</v>
+      </c>
+      <c r="B68" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>99</v>
+      </c>
+      <c r="B69" t="s">
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>